<commit_message>
Fix Balance Check: include pre-period Retained Earnings equity entries when no stmt_header
Co-authored-by: blufinLabs <45982520+blufinLabs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/reports/blufin_financial_statements.xlsx
+++ b/finance/reports/blufin_financial_statements.xlsx
@@ -4510,7 +4510,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>As of 2026-03-10</t>
+          <t>Period: 2025-01-01 to 2026-03-11</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4922,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Quarter Comparison: Current (2026-01-01 to 2026-03-10) vs Previous (2025-10-01 to 2025-12-31)</t>
+          <t>Quarter Comparison: Current (2026-01-01 to 2026-03-11) vs Previous (2025-10-01 to 2025-12-31)</t>
         </is>
       </c>
     </row>
@@ -5546,7 +5546,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>As of 2026-03-10</t>
+          <t>As of 2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix balance check by including Retained Earnings equity entries in ledger-only path
Co-authored-by: blufinLabs <45982520+blufinLabs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/reports/blufin_financial_statements.xlsx
+++ b/finance/reports/blufin_financial_statements.xlsx
@@ -82,10 +82,10 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -263,12 +263,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$L$11:$L$23</f>
+              <f>'Summary'!$L$11:$L$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$O$11:$O$23</f>
+              <f>'Summary'!$O$11:$O$26</f>
             </numRef>
           </val>
         </ser>
@@ -295,12 +295,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$L$11:$L$23</f>
+              <f>'Summary'!$L$11:$L$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$P$11:$P$23</f>
+              <f>'Summary'!$P$11:$P$26</f>
             </numRef>
           </val>
         </ser>
@@ -4479,13 +4479,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
     <col width="2" customWidth="1" min="7" max="7"/>
@@ -4495,7 +4495,7 @@
     <col width="2" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
   </cols>
@@ -4510,7 +4510,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Period: 2025-01-01 to 2025-12-31</t>
+          <t>Period: 2025-01-01 to 2026-03-11</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Beginning balance (2025-01-01)</t>
+          <t>Beginning balance as of 12/31/2024</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -4540,31 +4540,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total credits (period)</t>
+          <t>Total credits</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>89988.27</v>
+        <v>90176.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total debits (period)</t>
+          <t>Total debits</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>-66810.39999999999</v>
+        <v>-86680.53999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ending balance (2025-12-31)</t>
+          <t>Ending balance as of 03/11/2026</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>35508.23000000001</v>
+        <v>15826.45</v>
       </c>
     </row>
     <row r="9"/>
@@ -4867,14 +4867,62 @@
         <v>64248.66</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
+    <row r="24">
+      <c r="L24" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>5921.2</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>89526.53</v>
+      </c>
+      <c r="P24" s="3" t="n">
+        <v>70169.86</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="L25" s="4" t="n">
+        <v>46054</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>12770.4</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>89526.53</v>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>82940.26000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>990.1800000000001</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>89526.53</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>83930.44</v>
+      </c>
+    </row>
     <row r="27"/>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Quarter Comparison: Current (2025-10-01 to 2025-12-31) vs Previous (2025-07-01 to 2025-09-30)</t>
+          <t>Quarter Comparison: Current (2026-01-01 to 2026-03-11) vs Previous (2025-10-01 to 2025-12-31)</t>
         </is>
       </c>
     </row>
@@ -4917,108 +4965,108 @@
       <c r="P29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Bank Fees</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Electronic Components</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>1602.34</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>1217.6</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>0.3159822601839682</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Labor (Consulting)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>25100</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>-0.4023904382470119</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Machining/Fabrication</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>1248.64</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>15115.44</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>-0.9173930762187539</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mechanical Components</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>500.87</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>868.39</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>-0.42321998180541</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Misc Income</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="E30" s="6" t="n">
+      <c r="D34" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" s="8" t="n">
         <v>-1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Consulting Revenue</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>77369.7</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Electronic Components</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>1217.6</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>298.83</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>3.07455744068534</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Labor (Consulting)</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="n">
-        <v>25100</v>
-      </c>
-      <c r="D33" s="8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E33" s="9" t="n">
-        <v>4.02</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Machining/Fabrication</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>15115.44</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v/>
       </c>
     </row>
     <row r="35">
@@ -5029,16 +5077,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mechanical Components</t>
+          <t>Office Expenses</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>868.39</v>
+        <v>517.97</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="E35" s="9" t="n">
         <v/>
       </c>
     </row>
@@ -5050,38 +5098,38 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Misc Expense</t>
+          <t>Optical Components</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0</v>
+        <v>586.62</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>-1</v>
+        <v>5163.77</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>-0.8863969541633342</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Misc Income</t>
+          <t>Shipping Fees</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>100</v>
+        <v>26.34</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v/>
+        <v>36.64</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>-0.2811135371179039</v>
       </c>
     </row>
     <row r="38">
@@ -5092,17 +5140,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Optical Components</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>5163.77</v>
+        <v>160</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v/>
+        <v>3161.55</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>-0.9493919121949677</v>
       </c>
     </row>
     <row r="39">
@@ -5113,101 +5161,80 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Shipping Fees</t>
+          <t>Subscriptions and Memberships</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>36.64</v>
+        <v>39</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>84.36</v>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>-0.5656709340919868</v>
+        <v>0</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Software</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>3161.55</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>4512.01</v>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>-0.2993034146644178</v>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Total Income</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D41" s="8" t="n">
-        <v>77369.7</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>19681.78</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>50663.39</v>
       </c>
       <c r="E41" s="9" t="n">
-        <v>-0.9987075043589415</v>
+        <v>-0.6115186922943766</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Expenses</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Total Expenses</t>
+          <t>Net Income</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>50663.39</v>
+        <v>-19681.78</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>9955.200000000001</v>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>4.089138339762134</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
         <v>-50563.39</v>
       </c>
-      <c r="D43" s="3" t="n">
-        <v>67414.5</v>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>-1.750037306514177</v>
+      <c r="E42" s="9" t="n">
+        <v>-0.6107503867917083</v>
       </c>
     </row>
   </sheetData>
@@ -5222,11 +5249,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -5243,7 +5270,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-12-31</t>
+          <t>2025-01-01 to 2026-03-11</t>
         </is>
       </c>
     </row>
@@ -5319,7 +5346,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2033.44</v>
+        <v>3635.78</v>
       </c>
     </row>
     <row r="7">
@@ -5334,7 +5361,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>32100</v>
+        <v>47100</v>
       </c>
     </row>
     <row r="8">
@@ -5349,7 +5376,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>15115.44</v>
+        <v>16364.08</v>
       </c>
     </row>
     <row r="9">
@@ -5364,7 +5391,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>868.39</v>
+        <v>1369.26</v>
       </c>
     </row>
     <row r="10">
@@ -5390,11 +5417,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Optical Components</t>
+          <t>Office Expenses</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>5793.58</v>
+        <v>517.97</v>
       </c>
     </row>
     <row r="12">
@@ -5405,11 +5432,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Shipping Fees</t>
+          <t>Optical Components</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>186.25</v>
+        <v>6380.2</v>
       </c>
     </row>
     <row r="13">
@@ -5420,11 +5447,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Shipping Fees</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>8091.56</v>
+        <v>212.59</v>
       </c>
     </row>
     <row r="14">
@@ -5435,26 +5462,56 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Total Expenses</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>64248.66</v>
+        <v>8251.559999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Subscriptions and Memberships</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>83930.44</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Net Income</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
-        <v>25277.87</v>
+      <c r="C17" s="3" t="n">
+        <v>5596.089999999997</v>
       </c>
     </row>
   </sheetData>
@@ -5473,7 +5530,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5489,7 +5546,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>As of 2025-12-31</t>
+          <t>As of 2026-03-11</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5562,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>35508.23000000001</v>
+        <v>15826.45</v>
       </c>
     </row>
     <row r="3">
@@ -5520,7 +5577,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>35508.23000000001</v>
+        <v>15826.45</v>
       </c>
     </row>
     <row r="4">
@@ -5565,7 +5622,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0</v>
+        <v>12330.36</v>
       </c>
     </row>
     <row r="7">
@@ -5580,7 +5637,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>25277.87</v>
+        <v>5596.089999999997</v>
       </c>
     </row>
     <row r="8">
@@ -5595,7 +5652,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>23177.87</v>
+        <v>15826.45</v>
       </c>
     </row>
     <row r="9">
@@ -5610,7 +5667,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>12330.36000000001</v>
+        <v>3.637978807091713e-12</v>
       </c>
     </row>
   </sheetData>
@@ -5645,7 +5702,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Through 2025-12-31</t>
+          <t>Through 2026-03-11</t>
         </is>
       </c>
     </row>
@@ -5661,7 +5718,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>25277.87</v>
+        <v>5596.089999999997</v>
       </c>
     </row>
     <row r="3">
@@ -5706,7 +5763,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>89988.27</v>
+        <v>90176.63</v>
       </c>
     </row>
     <row r="6">
@@ -5721,7 +5778,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>-66810.39999999999</v>
+        <v>-86680.53999999999</v>
       </c>
     </row>
     <row r="7">
@@ -5736,7 +5793,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>25277.87</v>
+        <v>5596.089999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>